<commit_message>
Save file with complete task
</commit_message>
<xml_diff>
--- a/masterplan_hoja_de_ruta.xlsx
+++ b/masterplan_hoja_de_ruta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ro-ma\Documents\Github\Agenda-for-dummies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{116C35A8-B788-4ACF-B9C6-C7456248C9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1C2BEC-8E79-43F5-BB62-38F6CA0BBE57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1026,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1218,28 +1218,10 @@
     <xf numFmtId="0" fontId="29" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1631,66 +1613,66 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="28" t="s">
+      <c r="G6" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="31" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="35" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="37" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="39" t="s">
+      <c r="I7" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="40" t="s">
+      <c r="J7" s="31" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4305,7 +4287,7 @@
         <v>194</v>
       </c>
       <c r="E5" s="62">
-        <f t="shared" ref="E5:E20" si="0">D6-C6</f>
+        <f>D5-C5</f>
         <v>0</v>
       </c>
       <c r="F5" s="63" t="s">
@@ -4319,263 +4301,267 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="60" t="s">
         <v>197</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="B6" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67">
+      <c r="C6" s="61">
+        <v>46157</v>
+      </c>
+      <c r="D6" s="61">
+        <v>46158</v>
+      </c>
+      <c r="E6" s="62">
+        <f t="shared" ref="E6:E20" si="0">D6-C6</f>
+        <v>1</v>
+      </c>
+      <c r="F6" s="63"/>
+      <c r="G6" s="64" t="s">
+        <v>199</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>200</v>
+      </c>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F6" s="68"/>
-      <c r="G6" s="69" t="s">
-        <v>199</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="70" t="s">
-        <v>197</v>
-      </c>
-      <c r="B7" s="35" t="s">
-        <v>200</v>
-      </c>
-      <c r="C7" s="71"/>
-      <c r="D7" s="71"/>
-      <c r="E7" s="72">
+      <c r="F7" s="67"/>
+      <c r="G7" s="68"/>
+      <c r="H7" s="66"/>
+    </row>
+    <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="65" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F7" s="73"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="71"/>
-    </row>
-    <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="70" t="s">
+      <c r="F8" s="67"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="66"/>
+    </row>
+    <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="35" t="s">
-        <v>201</v>
-      </c>
-      <c r="C8" s="71"/>
-      <c r="D8" s="71"/>
-      <c r="E8" s="72">
+      <c r="B9" s="35" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="73"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="71"/>
-    </row>
-    <row r="9" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="70" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="35" t="s">
-        <v>202</v>
-      </c>
-      <c r="C9" s="71"/>
-      <c r="D9" s="71"/>
-      <c r="E9" s="72">
+      <c r="F9" s="67"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="66"/>
+    </row>
+    <row r="10" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="65" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="35" t="s">
+        <v>203</v>
+      </c>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="71"/>
-    </row>
-    <row r="10" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="70" t="s">
+      <c r="F10" s="67"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="66"/>
+    </row>
+    <row r="11" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="35" t="s">
-        <v>203</v>
-      </c>
-      <c r="C10" s="71"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="72">
+      <c r="B11" s="35" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F10" s="73"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="71"/>
-    </row>
-    <row r="11" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="70" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="35" t="s">
-        <v>204</v>
-      </c>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="72">
+      <c r="F11" s="67"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="66"/>
+    </row>
+    <row r="12" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="65" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F11" s="73"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="71"/>
-    </row>
-    <row r="12" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="70" t="s">
+      <c r="F12" s="67"/>
+      <c r="G12" s="68"/>
+      <c r="H12" s="66"/>
+    </row>
+    <row r="13" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="35" t="s">
-        <v>205</v>
-      </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="72">
+      <c r="B13" s="35" t="s">
+        <v>206</v>
+      </c>
+      <c r="C13" s="66"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F12" s="73"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="71"/>
-    </row>
-    <row r="13" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="70" t="s">
+      <c r="F13" s="67"/>
+      <c r="G13" s="68"/>
+      <c r="H13" s="66"/>
+    </row>
+    <row r="14" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>206</v>
-      </c>
-      <c r="C13" s="71"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="72">
+      <c r="B14" s="35" t="s">
+        <v>207</v>
+      </c>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F13" s="73"/>
-      <c r="G13" s="74"/>
-      <c r="H13" s="71"/>
-    </row>
-    <row r="14" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="70" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>207</v>
-      </c>
-      <c r="C14" s="71"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="72">
+      <c r="F14" s="67"/>
+      <c r="G14" s="68"/>
+      <c r="H14" s="66"/>
+    </row>
+    <row r="15" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="65" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>208</v>
+      </c>
+      <c r="C15" s="66"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F14" s="73"/>
-      <c r="G14" s="74"/>
-      <c r="H14" s="71"/>
-    </row>
-    <row r="15" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="70" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>208</v>
-      </c>
-      <c r="C15" s="71"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="72">
+      <c r="F15" s="67"/>
+      <c r="G15" s="68"/>
+      <c r="H15" s="66"/>
+    </row>
+    <row r="16" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="65" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>209</v>
+      </c>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F15" s="73"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="71"/>
-    </row>
-    <row r="16" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="70" t="s">
+      <c r="F16" s="67"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="66"/>
+    </row>
+    <row r="17" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="65" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="35" t="s">
-        <v>209</v>
-      </c>
-      <c r="C16" s="71"/>
-      <c r="D16" s="71"/>
-      <c r="E16" s="72">
+      <c r="B17" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F16" s="73"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="71"/>
-    </row>
-    <row r="17" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="70" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="C17" s="71"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="72">
+      <c r="F17" s="67"/>
+      <c r="G17" s="68"/>
+      <c r="H17" s="66"/>
+    </row>
+    <row r="18" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>211</v>
+      </c>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="73"/>
-      <c r="G17" s="74"/>
-      <c r="H17" s="71"/>
-    </row>
-    <row r="18" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="70" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="35" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" s="71"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="72">
+      <c r="F18" s="67"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="66"/>
+    </row>
+    <row r="19" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="65" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="C19" s="66"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="73"/>
-      <c r="G18" s="74"/>
-      <c r="H18" s="71"/>
-    </row>
-    <row r="19" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="70" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>212</v>
-      </c>
-      <c r="C19" s="71"/>
-      <c r="D19" s="71"/>
-      <c r="E19" s="72">
+      <c r="F19" s="67"/>
+      <c r="G19" s="68"/>
+      <c r="H19" s="66"/>
+    </row>
+    <row r="20" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="65" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="35" t="s">
+        <v>213</v>
+      </c>
+      <c r="C20" s="66"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F19" s="73"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="71"/>
-    </row>
-    <row r="20" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="70" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" s="35" t="s">
-        <v>213</v>
-      </c>
-      <c r="C20" s="71"/>
-      <c r="D20" s="71"/>
-      <c r="E20" s="72">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F20" s="73"/>
-      <c r="G20" s="74"/>
-      <c r="H20" s="71"/>
+      <c r="F20" s="67"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="66"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="12"/>

</xml_diff>